<commit_message>
feat: varredura e atualizacao ate 10/10 com 30 lojas e 2030 pedidos recuperados e novo dia 10/10
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-08).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-08).xlsx
@@ -935,10 +935,10 @@
     <t>214</t>
   </si>
   <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>R$ 4.567,90</t>
+    <t>34</t>
+  </si>
+  <si>
+    <t>R$ 4.558,43</t>
   </si>
   <si>
     <t>51.2</t>
@@ -947,7 +947,7 @@
     <t>32.6</t>
   </si>
   <si>
-    <t>4.99</t>
+    <t>5.00</t>
   </si>
   <si>
     <t>18.6</t>
@@ -959,7 +959,7 @@
     <t>6.0</t>
   </si>
   <si>
-    <t>43.1%</t>
+    <t>43.2%</t>
   </si>
   <si>
     <t>20.1%</t>
@@ -30839,7 +30839,7 @@
         <v>19951</v>
       </c>
       <c r="B199" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C199" s="4">
         <v>51</v>
@@ -30869,14 +30869,26 @@
         <v>58</v>
       </c>
       <c r="L199" s="4"/>
-      <c r="M199" s="5"/>
-      <c r="N199" s="6"/>
+      <c r="M199" s="5">
+        <v>2873.54</v>
+      </c>
+      <c r="N199" s="6">
+        <v>34</v>
+      </c>
       <c r="O199" s="6"/>
-      <c r="P199" s="7"/>
-      <c r="Q199" s="8"/>
-      <c r="R199" s="8"/>
+      <c r="P199" s="7">
+        <v>5.4600999999999997</v>
+      </c>
+      <c r="Q199" s="8">
+        <v>17.853124999999999</v>
+      </c>
+      <c r="R199" s="8">
+        <v>4.8770812499999998</v>
+      </c>
       <c r="S199" s="8"/>
-      <c r="T199" s="9"/>
+      <c r="T199" s="9">
+        <v>0.25</v>
+      </c>
       <c r="U199" s="9"/>
       <c r="V199" s="9"/>
       <c r="W199" s="9"/>

</xml_diff>